<commit_message>
C2 (part 1): move 02 functions to 模型函数.R and add 04 script
- Move the function definitions of 02 (score to rolling_predict, old
  lines 15-134) verbatim into R研究/模型函数.R; 02 now sources it. The
  expanded expressions are identical to the original 02, so 02 is not
  re-run.
- 03 sources 模型函数.R and reports mean errors as actual minus forecast
  (positive = under-prediction), matching table 9 of the revised draft;
  re-run, all other values unchanged.
- Add 04_9月检验与实际预测.R (September check, 2026-10-01 forecast,
  October path); its run is in progress and outputs follow in the next
  commit. Checkpoints in results/04_中间结果/ are git-ignored.
- Plan: record that 03 matches tables 9-10 of the revised draft.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LzekgcBgpeFtnjtKcg5s5Y
</commit_message>
<xml_diff>
--- a/R研究/results/补充检验结果.xlsx
+++ b/R研究/results/补充检验结果.xlsx
@@ -1226,7 +1226,7 @@
         <v>3.544619042727959E-10</v>
       </c>
       <c r="J2">
-        <v>-8.092109910836761</v>
+        <v>8.092109910836761</v>
       </c>
     </row>
     <row r="3">
@@ -1260,7 +1260,7 @@
         <v>5.023342852794599E-10</v>
       </c>
       <c r="J3">
-        <v>-0.7695276063100123</v>
+        <v>0.7695276063100123</v>
       </c>
     </row>
     <row r="4">
@@ -1294,7 +1294,7 @@
         <v>0.00140778682862408</v>
       </c>
       <c r="J4">
-        <v>-2.480643621106234</v>
+        <v>2.480643621106234</v>
       </c>
     </row>
     <row r="5">
@@ -1328,7 +1328,7 @@
         <v>0.004615600331127179</v>
       </c>
       <c r="J5">
-        <v>-10.6404822081452</v>
+        <v>10.6404822081452</v>
       </c>
     </row>
     <row r="6">
@@ -1362,7 +1362,7 @@
         <v>6.439293542825908E-15</v>
       </c>
       <c r="J6">
-        <v>-25.94754521351007</v>
+        <v>25.94754521351007</v>
       </c>
     </row>
     <row r="7">
@@ -1396,7 +1396,7 @@
         <v>0.09440990408259398</v>
       </c>
       <c r="J7">
-        <v>-8.89555410713433</v>
+        <v>8.89555410713433</v>
       </c>
     </row>
     <row r="8">
@@ -1430,7 +1430,7 @@
         <v>3.831596151471217E-10</v>
       </c>
       <c r="J8">
-        <v>-4.970239760159457</v>
+        <v>4.970239760159457</v>
       </c>
     </row>
     <row r="9">
@@ -1464,7 +1464,7 @@
         <v>0.0001478005098061175</v>
       </c>
       <c r="J9">
-        <v>-9.331958218265703</v>
+        <v>9.331958218265703</v>
       </c>
     </row>
   </sheetData>
@@ -3149,11 +3149,11 @@
         <v>243</v>
       </c>
       <c r="D17">
-        <v>-9.331958218265703</v>
+        <v>9.331958218265703</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Prediction minus actual, SGD/MWh; negative = under-prediction on average</t>
+          <t>Actual minus prediction, SGD/MWh; positive = under-prediction on average</t>
         </is>
       </c>
     </row>

</xml_diff>